<commit_message>
Add IMU orientation module with main implementation and update CMake configuration; enhance button LED feedback
</commit_message>
<xml_diff>
--- a/Docs/Pi500_Cpp_Lab_Tracker filled.xlsx
+++ b/Docs/Pi500_Cpp_Lab_Tracker filled.xlsx
@@ -4,7 +4,7 @@
   <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="4"/>
+    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet r:id="rId1" sheetId="1" name="Dashboard"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="362">
   <si>
     <t>REVIEW PROMPTS — BRING THESE, NOT THE BLANKS</t>
   </si>
@@ -723,6 +723,9 @@
     <t>What do you lose vs a single libgpiod request object on this circuit?</t>
   </si>
   <si>
+    <t xml:space="preserve">The question is poorly phrased. You lose the ability to track changes in  several parallel components. But not relevant to this circuit bc there are just two components:  a button (input) and an LED (output, state machine). </t>
+  </si>
+  <si>
     <t>Range 100: duty for ~50%? Soft PWM vs hardware PWM — what differs?</t>
   </si>
   <si>
@@ -801,6 +804,15 @@
     <t>Soon?</t>
   </si>
   <si>
+    <t>Coded to detect a button edge change</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>Dunno</t>
+  </si>
+  <si>
     <t>Tip: if a sitting spans two lessons, log two rows. The Lessons sheet sums hours by lesson number.</t>
   </si>
   <si>
@@ -895,9 +907,6 @@
   </si>
   <si>
     <t>LED on BCM 18</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>RGB LED</t>
@@ -1125,7 +1134,7 @@
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="166" formatCode="#,##0%"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1144,6 +1153,12 @@
       <i/>
       <sz val="10"/>
       <color rgb="FF0e7c7b"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1169,7 +1184,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -1389,325 +1404,322 @@
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="9" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="10" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="9" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="9" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="10" applyFont="1" fillId="9" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="12" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="13" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="9" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="4" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="16" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="8" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="3" applyBorder="1" fontId="3" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="6" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="13" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="14" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="15" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="2" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="7" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="16" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="17" applyFont="1" fillId="10" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="18" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
@@ -1716,77 +1728,80 @@
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="19" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="20" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="20" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="11" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="21" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="12" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="21" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="5" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="22" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="21" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="22" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="21" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="22" applyFont="1" fillId="8" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="5" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="7" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="4" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="6" applyFont="1" fillId="6" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="8" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="1" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
-    <xf xfId="0" numFmtId="166" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2093,77 +2108,77 @@
   <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="134" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="37" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="37" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="135" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="134" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="49" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="20" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="38" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="38" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="134" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="135" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="50" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="16.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
       <c r="A1" s="84" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B1" s="85"/>
       <c r="C1" s="85"/>
       <c r="D1" s="86"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="87"/>
+      <c r="E1" s="87"/>
+      <c r="F1" s="84"/>
       <c r="G1" s="88"/>
-      <c r="H1" s="87"/>
+      <c r="H1" s="84"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
       <c r="A2" s="89" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B2" s="90"/>
       <c r="C2" s="90"/>
       <c r="D2" s="91"/>
-      <c r="E2" s="89"/>
-      <c r="F2" s="92"/>
+      <c r="E2" s="92"/>
+      <c r="F2" s="89"/>
       <c r="G2" s="93"/>
-      <c r="H2" s="92"/>
+      <c r="H2" s="89"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
       <c r="A3" s="94" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B3" s="95"/>
       <c r="C3" s="95"/>
       <c r="D3" s="96"/>
-      <c r="E3" s="94"/>
-      <c r="F3" s="97"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="94"/>
       <c r="G3" s="98"/>
-      <c r="H3" s="97"/>
+      <c r="H3" s="94"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
       <c r="A4" s="99"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
       <c r="D4" s="100"/>
       <c r="E4" s="99"/>
       <c r="F4" s="13"/>
-      <c r="G4" s="40"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
       <c r="A5" s="101" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B5" s="102"/>
       <c r="C5" s="103" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D5" s="104"/>
       <c r="E5" s="105" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F5" s="106"/>
       <c r="G5" s="107" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="H5" s="108"/>
     </row>
@@ -2187,49 +2202,49 @@
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="99"/>
-      <c r="B7" s="29"/>
-      <c r="C7" s="29"/>
+      <c r="B7" s="30"/>
+      <c r="C7" s="30"/>
       <c r="D7" s="100"/>
       <c r="E7" s="99"/>
       <c r="F7" s="13"/>
-      <c r="G7" s="40"/>
+      <c r="G7" s="41"/>
       <c r="H7" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
-      <c r="A8" s="113" t="s">
-        <v>337</v>
-      </c>
-      <c r="B8" s="114"/>
-      <c r="C8" s="114"/>
-      <c r="D8" s="115"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="44"/>
-      <c r="G8" s="45"/>
-      <c r="H8" s="44"/>
+      <c r="A8" s="45" t="s">
+        <v>340</v>
+      </c>
+      <c r="B8" s="113"/>
+      <c r="C8" s="113"/>
+      <c r="D8" s="114"/>
+      <c r="E8" s="115"/>
+      <c r="F8" s="45"/>
+      <c r="G8" s="46"/>
+      <c r="H8" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="116" t="s">
-        <v>261</v>
-      </c>
-      <c r="B9" s="30" t="s">
-        <v>338</v>
-      </c>
-      <c r="C9" s="30" t="s">
-        <v>274</v>
-      </c>
-      <c r="D9" s="117" t="s">
-        <v>339</v>
-      </c>
-      <c r="E9" s="116" t="s">
+      <c r="A9" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="B9" s="31" t="s">
+        <v>341</v>
+      </c>
+      <c r="C9" s="31" t="s">
+        <v>278</v>
+      </c>
+      <c r="D9" s="116" t="s">
+        <v>342</v>
+      </c>
+      <c r="E9" s="117" t="s">
         <v>190</v>
       </c>
       <c r="F9" s="13"/>
-      <c r="G9" s="40"/>
+      <c r="G9" s="41"/>
       <c r="H9" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
       <c r="A10" s="118" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B10" s="119">
         <v>11</v>
@@ -2244,12 +2259,12 @@
         <f>IF(C10=B10,"Unit cleared",IF(C10=0,"Not started","In progress"))</f>
       </c>
       <c r="F10" s="13"/>
-      <c r="G10" s="40"/>
+      <c r="G10" s="41"/>
       <c r="H10" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
       <c r="A11" s="122" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B11" s="123">
         <v>4</v>
@@ -2264,39 +2279,39 @@
         <f>IF(C11=B11,"Unit cleared",IF(C11=0,"Not started","In progress"))</f>
       </c>
       <c r="F11" s="13"/>
-      <c r="G11" s="40"/>
+      <c r="G11" s="41"/>
       <c r="H11" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
       <c r="A12" s="99"/>
-      <c r="B12" s="29"/>
-      <c r="C12" s="29"/>
+      <c r="B12" s="30"/>
+      <c r="C12" s="30"/>
       <c r="D12" s="100"/>
       <c r="E12" s="99"/>
       <c r="F12" s="13"/>
-      <c r="G12" s="40"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="113" t="s">
-        <v>342</v>
-      </c>
-      <c r="B13" s="114"/>
-      <c r="C13" s="114"/>
-      <c r="D13" s="115"/>
-      <c r="E13" s="113"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="44"/>
+      <c r="A13" s="45" t="s">
+        <v>345</v>
+      </c>
+      <c r="B13" s="113"/>
+      <c r="C13" s="113"/>
+      <c r="D13" s="114"/>
+      <c r="E13" s="115"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
       <c r="A14" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B14" s="55" t="s">
-        <v>344</v>
-      </c>
-      <c r="C14" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B14" s="56" t="s">
+        <v>347</v>
+      </c>
+      <c r="C14" s="56"/>
       <c r="D14" s="127"/>
       <c r="E14" s="125"/>
       <c r="F14" s="10"/>
@@ -2305,12 +2320,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
       <c r="A15" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B15" s="55" t="s">
-        <v>345</v>
-      </c>
-      <c r="C15" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B15" s="56" t="s">
+        <v>348</v>
+      </c>
+      <c r="C15" s="56"/>
       <c r="D15" s="127"/>
       <c r="E15" s="125"/>
       <c r="F15" s="10"/>
@@ -2319,12 +2334,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
       <c r="A16" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B16" s="55" t="s">
         <v>346</v>
       </c>
-      <c r="C16" s="55"/>
+      <c r="B16" s="56" t="s">
+        <v>349</v>
+      </c>
+      <c r="C16" s="56"/>
       <c r="D16" s="127"/>
       <c r="E16" s="125"/>
       <c r="F16" s="10"/>
@@ -2333,12 +2348,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
       <c r="A17" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B17" s="55" t="s">
-        <v>347</v>
-      </c>
-      <c r="C17" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B17" s="56" t="s">
+        <v>350</v>
+      </c>
+      <c r="C17" s="56"/>
       <c r="D17" s="127"/>
       <c r="E17" s="125"/>
       <c r="F17" s="10"/>
@@ -2347,12 +2362,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
       <c r="A18" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B18" s="55" t="s">
-        <v>348</v>
-      </c>
-      <c r="C18" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B18" s="56" t="s">
+        <v>351</v>
+      </c>
+      <c r="C18" s="56"/>
       <c r="D18" s="127"/>
       <c r="E18" s="125"/>
       <c r="F18" s="10"/>
@@ -2361,12 +2376,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="21.75">
       <c r="A19" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B19" s="55" t="s">
-        <v>349</v>
-      </c>
-      <c r="C19" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B19" s="56" t="s">
+        <v>352</v>
+      </c>
+      <c r="C19" s="56"/>
       <c r="D19" s="127"/>
       <c r="E19" s="125"/>
       <c r="F19" s="10"/>
@@ -2375,12 +2390,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="21.75">
       <c r="A20" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B20" s="55" t="s">
-        <v>350</v>
-      </c>
-      <c r="C20" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B20" s="56" t="s">
+        <v>353</v>
+      </c>
+      <c r="C20" s="56"/>
       <c r="D20" s="127"/>
       <c r="E20" s="125"/>
       <c r="F20" s="10"/>
@@ -2389,12 +2404,12 @@
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="21.75">
       <c r="A21" s="126" t="s">
-        <v>343</v>
-      </c>
-      <c r="B21" s="55" t="s">
-        <v>351</v>
-      </c>
-      <c r="C21" s="55"/>
+        <v>346</v>
+      </c>
+      <c r="B21" s="56" t="s">
+        <v>354</v>
+      </c>
+      <c r="C21" s="56"/>
       <c r="D21" s="127"/>
       <c r="E21" s="125"/>
       <c r="F21" s="10"/>
@@ -2403,44 +2418,44 @@
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="21.75">
       <c r="A22" s="99"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="29"/>
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
       <c r="D22" s="100"/>
       <c r="E22" s="99"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="40"/>
+      <c r="G22" s="41"/>
       <c r="H22" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="21.75">
-      <c r="A23" s="113" t="s">
-        <v>352</v>
-      </c>
-      <c r="B23" s="114"/>
-      <c r="C23" s="114"/>
-      <c r="D23" s="115"/>
-      <c r="E23" s="113"/>
-      <c r="F23" s="44"/>
-      <c r="G23" s="45"/>
-      <c r="H23" s="44"/>
+      <c r="A23" s="45" t="s">
+        <v>355</v>
+      </c>
+      <c r="B23" s="113"/>
+      <c r="C23" s="113"/>
+      <c r="D23" s="114"/>
+      <c r="E23" s="115"/>
+      <c r="F23" s="45"/>
+      <c r="G23" s="46"/>
+      <c r="H23" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
-      <c r="A24" s="128" t="s">
-        <v>353</v>
-      </c>
-      <c r="B24" s="129"/>
-      <c r="C24" s="129"/>
-      <c r="D24" s="130"/>
-      <c r="E24" s="128"/>
-      <c r="F24" s="34"/>
+      <c r="A24" s="35" t="s">
+        <v>356</v>
+      </c>
+      <c r="B24" s="128"/>
+      <c r="C24" s="128"/>
+      <c r="D24" s="129"/>
+      <c r="E24" s="130"/>
+      <c r="F24" s="35"/>
       <c r="G24" s="131"/>
-      <c r="H24" s="34"/>
+      <c r="H24" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
-      <c r="A25" s="125" t="s">
-        <v>354</v>
-      </c>
-      <c r="B25" s="55"/>
-      <c r="C25" s="55"/>
+      <c r="A25" s="10" t="s">
+        <v>357</v>
+      </c>
+      <c r="B25" s="56"/>
+      <c r="C25" s="56"/>
       <c r="D25" s="127"/>
       <c r="E25" s="125"/>
       <c r="F25" s="10"/>
@@ -2448,23 +2463,23 @@
       <c r="H25" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21.75">
-      <c r="A26" s="128" t="s">
-        <v>355</v>
-      </c>
-      <c r="B26" s="129"/>
-      <c r="C26" s="129"/>
-      <c r="D26" s="130"/>
-      <c r="E26" s="128"/>
-      <c r="F26" s="34"/>
+      <c r="A26" s="35" t="s">
+        <v>358</v>
+      </c>
+      <c r="B26" s="128"/>
+      <c r="C26" s="128"/>
+      <c r="D26" s="129"/>
+      <c r="E26" s="130"/>
+      <c r="F26" s="35"/>
       <c r="G26" s="131"/>
-      <c r="H26" s="34"/>
+      <c r="H26" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21.75">
-      <c r="A27" s="125" t="s">
-        <v>356</v>
-      </c>
-      <c r="B27" s="55"/>
-      <c r="C27" s="55"/>
+      <c r="A27" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="B27" s="56"/>
+      <c r="C27" s="56"/>
       <c r="D27" s="127"/>
       <c r="E27" s="125"/>
       <c r="F27" s="10"/>
@@ -2472,35 +2487,35 @@
       <c r="H27" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="21.75">
-      <c r="A28" s="128" t="s">
-        <v>357</v>
-      </c>
-      <c r="B28" s="129"/>
-      <c r="C28" s="129"/>
-      <c r="D28" s="130"/>
-      <c r="E28" s="128"/>
-      <c r="F28" s="34"/>
+      <c r="A28" s="35" t="s">
+        <v>360</v>
+      </c>
+      <c r="B28" s="128"/>
+      <c r="C28" s="128"/>
+      <c r="D28" s="129"/>
+      <c r="E28" s="130"/>
+      <c r="F28" s="35"/>
       <c r="G28" s="131"/>
-      <c r="H28" s="34"/>
+      <c r="H28" s="35"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="21.75">
       <c r="A29" s="99"/>
-      <c r="B29" s="29"/>
-      <c r="C29" s="29"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
       <c r="D29" s="100"/>
       <c r="E29" s="99"/>
       <c r="F29" s="13"/>
-      <c r="G29" s="40"/>
+      <c r="G29" s="41"/>
       <c r="H29" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="21.75">
-      <c r="A30" s="132" t="s">
-        <v>358</v>
-      </c>
-      <c r="B30" s="36"/>
-      <c r="C30" s="36"/>
-      <c r="D30" s="133"/>
-      <c r="E30" s="132"/>
+      <c r="A30" s="19" t="s">
+        <v>361</v>
+      </c>
+      <c r="B30" s="37"/>
+      <c r="C30" s="37"/>
+      <c r="D30" s="132"/>
+      <c r="E30" s="133"/>
       <c r="F30" s="19"/>
       <c r="G30" s="71"/>
       <c r="H30" s="19"/>
@@ -2548,55 +2563,55 @@
   <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="37" width="5.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="2.2907142857142855" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="49" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="20" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="37" width="15.862142857142858" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="11" max="11" style="20" width="15.862142857142858" customWidth="1" bestFit="1" hidden="1"/>
-    <col min="12" max="12" style="20" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="38" width="5.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="2.2907142857142855" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="50" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="73" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="38" width="15.862142857142858" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="11" max="11" style="12" width="15.862142857142858" customWidth="1" bestFit="1" hidden="1"/>
+    <col min="12" max="12" style="12" width="14.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
-      <c r="A1" s="25" t="s">
-        <v>255</v>
+      <c r="A1" s="26" t="s">
+        <v>259</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="38"/>
+      <c r="G1" s="39"/>
       <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="25"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="26"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
-      <c r="A2" s="26" t="s">
-        <v>256</v>
+      <c r="A2" s="27" t="s">
+        <v>260</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="39"/>
+      <c r="G2" s="40"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="26"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="27"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
       <c r="A3" s="74" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B3" s="75"/>
       <c r="C3" s="76">
@@ -2604,577 +2619,557 @@
       </c>
       <c r="D3" s="13"/>
       <c r="E3" s="77" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="F3" s="77"/>
       <c r="G3" s="62">
         <f>SUM(J8:J22)</f>
       </c>
       <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="29"/>
+      <c r="I3" s="78"/>
+      <c r="J3" s="30"/>
       <c r="K3" s="13"/>
       <c r="L3" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
-      <c r="A4" s="29"/>
+      <c r="A4" s="30"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
-      <c r="G4" s="40"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="29"/>
+      <c r="I4" s="78"/>
+      <c r="J4" s="30"/>
       <c r="K4" s="13"/>
       <c r="L4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
-      <c r="A5" s="29"/>
+      <c r="A5" s="30"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
-      <c r="G5" s="40"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="29"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="30"/>
       <c r="K5" s="13"/>
       <c r="L5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
-      <c r="A6" s="29"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
-      <c r="G6" s="40"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="29"/>
+      <c r="I6" s="78"/>
+      <c r="J6" s="30"/>
       <c r="K6" s="13"/>
       <c r="L6" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="66" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="G7" s="67" t="s">
         <v>190</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>266</v>
+        <v>269</v>
+      </c>
+      <c r="I7" s="68" t="s">
+        <v>270</v>
       </c>
       <c r="J7" s="66" t="s">
         <v>191</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>267</v>
+        <v>271</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
-      <c r="A8" s="31">
+      <c r="A8" s="32">
         <v>1</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>269</v>
+        <v>273</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>272</v>
+        <v>276</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>273</v>
-      </c>
-      <c r="G8" s="78" t="s">
-        <v>274</v>
-      </c>
-      <c r="H8" s="79" t="s">
+        <v>277</v>
+      </c>
+      <c r="G8" s="79" t="s">
+        <v>278</v>
+      </c>
+      <c r="H8" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="8" t="s">
-        <v>251</v>
-      </c>
-      <c r="J8" s="80">
+      <c r="I8" s="81" t="s">
+        <v>252</v>
+      </c>
+      <c r="J8" s="82">
         <v>1</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="L8" s="13" t="s">
         <v>48</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="32">
+      <c r="A9" s="33">
         <v>2</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="F9" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G9" s="81" t="s">
-        <v>274</v>
-      </c>
-      <c r="H9" s="79" t="s">
+      <c r="G9" s="83" t="s">
+        <v>278</v>
+      </c>
+      <c r="H9" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="I9" s="82">
+      <c r="I9" s="81">
         <v>46266</v>
       </c>
-      <c r="J9" s="29">
+      <c r="J9" s="30">
         <v>1</v>
       </c>
       <c r="K9" s="13"/>
       <c r="L9" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
-      <c r="A10" s="31">
+      <c r="A10" s="32">
         <v>3</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>270</v>
+        <v>274</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>280</v>
+        <v>284</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>281</v>
+        <v>285</v>
       </c>
       <c r="F10" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="G10" s="78" t="s">
+      <c r="G10" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H10" s="79" t="s">
+      <c r="H10" s="80" t="s">
         <v>48</v>
       </c>
-      <c r="I10" s="82"/>
-      <c r="J10" s="29"/>
+      <c r="I10" s="81">
+        <v>46268</v>
+      </c>
+      <c r="J10" s="30"/>
       <c r="K10" s="13"/>
       <c r="L10" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
-      <c r="A11" s="32">
+      <c r="A11" s="33">
         <v>4</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>282</v>
+        <v>286</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>283</v>
+        <v>287</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>284</v>
+        <v>288</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>285</v>
+        <v>289</v>
       </c>
       <c r="F11" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G11" s="81" t="s">
+      <c r="G11" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H11" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I11" s="82"/>
-      <c r="J11" s="29"/>
+      <c r="H11" s="80" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="81"/>
+      <c r="J11" s="30"/>
       <c r="K11" s="13"/>
       <c r="L11" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
-      <c r="A12" s="31">
+      <c r="A12" s="32">
         <v>5</v>
       </c>
       <c r="B12" s="7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>287</v>
       </c>
-      <c r="C12" s="7" t="s">
-        <v>283</v>
-      </c>
       <c r="D12" s="7" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="E12" s="7" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="F12" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="78" t="s">
+      <c r="G12" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H12" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I12" s="82"/>
-      <c r="J12" s="29"/>
+      <c r="H12" s="80"/>
+      <c r="I12" s="81"/>
+      <c r="J12" s="30"/>
       <c r="K12" s="13"/>
       <c r="L12" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="32">
+      <c r="A13" s="33">
         <v>6</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="F13" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="81" t="s">
+      <c r="G13" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H13" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I13" s="82"/>
-      <c r="J13" s="29"/>
+      <c r="H13" s="80"/>
+      <c r="I13" s="81"/>
+      <c r="J13" s="30"/>
       <c r="K13" s="13"/>
       <c r="L13" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
-      <c r="A14" s="31">
+      <c r="A14" s="32">
         <v>7</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="F14" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="G14" s="78" t="s">
+      <c r="G14" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H14" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I14" s="82"/>
-      <c r="J14" s="29"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="81"/>
+      <c r="J14" s="30"/>
       <c r="K14" s="13"/>
       <c r="L14" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
-      <c r="A15" s="32">
+      <c r="A15" s="33">
         <v>8</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="G15" s="81" t="s">
+        <v>305</v>
+      </c>
+      <c r="G15" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H15" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I15" s="82"/>
-      <c r="J15" s="29"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="81"/>
+      <c r="J15" s="30"/>
       <c r="K15" s="13"/>
       <c r="L15" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
-      <c r="A16" s="31">
+      <c r="A16" s="32">
         <v>9</v>
       </c>
       <c r="B16" s="7" t="s">
         <v>87</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="F16" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G16" s="78" t="s">
+      <c r="G16" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H16" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I16" s="82"/>
-      <c r="J16" s="29"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="81"/>
+      <c r="J16" s="30"/>
       <c r="K16" s="13"/>
       <c r="L16" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
-      <c r="A17" s="32">
+      <c r="A17" s="33">
         <v>10</v>
       </c>
       <c r="B17" s="10" t="s">
         <v>91</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F17" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G17" s="81" t="s">
+      <c r="G17" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H17" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I17" s="82"/>
-      <c r="J17" s="29"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="81"/>
+      <c r="J17" s="30"/>
       <c r="K17" s="13"/>
       <c r="L17" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
-      <c r="A18" s="31">
+      <c r="A18" s="32">
         <v>11</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F18" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="G18" s="78" t="s">
+      <c r="G18" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H18" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I18" s="82"/>
-      <c r="J18" s="29"/>
+      <c r="H18" s="80"/>
+      <c r="I18" s="81"/>
+      <c r="J18" s="30"/>
       <c r="K18" s="13"/>
       <c r="L18" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="21.75">
-      <c r="A19" s="32">
+      <c r="A19" s="33">
         <v>12</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>315</v>
-      </c>
-      <c r="G19" s="81" t="s">
+        <v>318</v>
+      </c>
+      <c r="G19" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H19" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I19" s="82"/>
-      <c r="J19" s="29"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="81"/>
+      <c r="J19" s="30"/>
       <c r="K19" s="13"/>
       <c r="L19" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="21.75">
-      <c r="A20" s="31">
+      <c r="A20" s="32">
         <v>13</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="E20" s="7" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="G20" s="78" t="s">
+      <c r="G20" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H20" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I20" s="82"/>
-      <c r="J20" s="29"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="81"/>
+      <c r="J20" s="30"/>
       <c r="K20" s="13"/>
       <c r="L20" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="21.75">
-      <c r="A21" s="32">
+      <c r="A21" s="33">
         <v>14</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="G21" s="81" t="s">
+        <v>326</v>
+      </c>
+      <c r="G21" s="83" t="s">
         <v>195</v>
       </c>
-      <c r="H21" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I21" s="82"/>
-      <c r="J21" s="29"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="81"/>
+      <c r="J21" s="30"/>
       <c r="K21" s="13"/>
       <c r="L21" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="21.75">
-      <c r="A22" s="31">
+      <c r="A22" s="32">
         <v>15</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E22" s="7" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>328</v>
-      </c>
-      <c r="G22" s="78" t="s">
+        <v>331</v>
+      </c>
+      <c r="G22" s="79" t="s">
         <v>195</v>
       </c>
-      <c r="H22" s="83" t="s">
-        <v>286</v>
-      </c>
-      <c r="I22" s="82"/>
-      <c r="J22" s="29"/>
+      <c r="H22" s="80"/>
+      <c r="I22" s="81"/>
+      <c r="J22" s="30"/>
       <c r="K22" s="13"/>
       <c r="L22" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="21.75">
-      <c r="A23" s="29"/>
+      <c r="A23" s="30"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
-      <c r="G23" s="40"/>
+      <c r="G23" s="41"/>
       <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="29"/>
+      <c r="I23" s="78"/>
+      <c r="J23" s="30"/>
       <c r="K23" s="13"/>
       <c r="L23" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
-      <c r="A24" s="36" t="s">
-        <v>329</v>
+      <c r="A24" s="37" t="s">
+        <v>332</v>
       </c>
       <c r="B24" s="19"/>
       <c r="C24" s="19"/>
@@ -3183,8 +3178,8 @@
       <c r="F24" s="19"/>
       <c r="G24" s="71"/>
       <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="36"/>
+      <c r="I24" s="72"/>
+      <c r="J24" s="37"/>
       <c r="K24" s="19"/>
       <c r="L24" s="19"/>
     </row>
@@ -3208,91 +3203,91 @@
   <dimension ref="A1:H50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="37" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="37" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="49" width="36.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="38" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="38" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="50" width="36.29071428571429" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="22.005" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="73" width="40.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="49" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="20" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="50" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="28.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
       <c r="A1" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="38"/>
+        <v>241</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="39"/>
       <c r="E1" s="1"/>
       <c r="F1" s="58"/>
-      <c r="G1" s="38"/>
+      <c r="G1" s="39"/>
       <c r="H1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
       <c r="A2" s="2" t="s">
-        <v>241</v>
-      </c>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="39"/>
+        <v>242</v>
+      </c>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="40"/>
       <c r="E2" s="2"/>
       <c r="F2" s="59"/>
-      <c r="G2" s="39"/>
+      <c r="G2" s="40"/>
       <c r="H2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
       <c r="A3" s="21" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B3" s="60">
         <f>COUNTA(A8:A200)</f>
       </c>
       <c r="C3" s="61" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D3" s="62">
         <f>SUM(G8:G200)</f>
       </c>
       <c r="E3" s="63" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F3" s="64">
         <f>IF(COUNTA(A8:A200)=0,"—",MAX(A8:A200))</f>
         <v>25568.791666666668</v>
       </c>
-      <c r="G3" s="40"/>
+      <c r="G3" s="41"/>
       <c r="H3" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
       <c r="A4" s="13"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="29"/>
-      <c r="D4" s="40"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="41"/>
       <c r="E4" s="13"/>
       <c r="F4" s="65"/>
-      <c r="G4" s="40"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
       <c r="A5" s="13"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="29"/>
-      <c r="D5" s="40"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="41"/>
       <c r="E5" s="13"/>
       <c r="F5" s="65"/>
-      <c r="G5" s="40"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
       <c r="A6" s="13"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="40"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="41"/>
       <c r="E6" s="13"/>
       <c r="F6" s="65"/>
-      <c r="G6" s="40"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
@@ -3300,545 +3295,561 @@
         <v>212</v>
       </c>
       <c r="B7" s="66" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C7" s="66" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D7" s="67" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F7" s="68" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G7" s="67" t="s">
         <v>191</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
       <c r="A8" s="7" t="s">
-        <v>251</v>
-      </c>
-      <c r="B8" s="56">
+        <v>252</v>
+      </c>
+      <c r="B8" s="57">
         <f>IF(A8="","",COUNTA($A$8:A8))</f>
       </c>
-      <c r="C8" s="56">
+      <c r="C8" s="57">
         <v>1</v>
       </c>
       <c r="D8" s="69" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F8" s="51"/>
+      <c r="F8" s="52"/>
       <c r="G8" s="69">
         <v>1.5</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="53"/>
-      <c r="B9" s="55">
+      <c r="A9" s="54">
+        <v>46266</v>
+      </c>
+      <c r="B9" s="56">
         <f>IF(A9="","",COUNTA($A$8:A9))</f>
       </c>
-      <c r="C9" s="55"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="53"/>
-      <c r="G9" s="70"/>
-      <c r="H9" s="10"/>
+      <c r="C9" s="56">
+        <v>2</v>
+      </c>
+      <c r="D9" s="70" t="s">
+        <v>255</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="F9" s="54" t="s">
+        <v>256</v>
+      </c>
+      <c r="G9" s="70">
+        <v>1.5</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>257</v>
+      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
-      <c r="A10" s="51"/>
-      <c r="B10" s="56">
+      <c r="A10" s="52">
+        <v>46268</v>
+      </c>
+      <c r="B10" s="57">
         <f>IF(A10="","",COUNTA($A$8:A10))</f>
       </c>
-      <c r="C10" s="56"/>
+      <c r="C10" s="57"/>
       <c r="D10" s="69"/>
       <c r="E10" s="7"/>
-      <c r="F10" s="51"/>
+      <c r="F10" s="52"/>
       <c r="G10" s="69"/>
       <c r="H10" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
-      <c r="A11" s="53"/>
-      <c r="B11" s="55">
+      <c r="A11" s="54"/>
+      <c r="B11" s="56">
         <f>IF(A11="","",COUNTA($A$8:A11))</f>
       </c>
-      <c r="C11" s="55"/>
+      <c r="C11" s="56"/>
       <c r="D11" s="70"/>
       <c r="E11" s="10"/>
-      <c r="F11" s="53"/>
+      <c r="F11" s="54"/>
       <c r="G11" s="70"/>
       <c r="H11" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
-      <c r="A12" s="51"/>
-      <c r="B12" s="56">
+      <c r="A12" s="52"/>
+      <c r="B12" s="57">
         <f>IF(A12="","",COUNTA($A$8:A12))</f>
       </c>
-      <c r="C12" s="56"/>
+      <c r="C12" s="57"/>
       <c r="D12" s="69"/>
       <c r="E12" s="7"/>
-      <c r="F12" s="51"/>
+      <c r="F12" s="52"/>
       <c r="G12" s="69"/>
       <c r="H12" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="53"/>
-      <c r="B13" s="55">
+      <c r="A13" s="54"/>
+      <c r="B13" s="56">
         <f>IF(A13="","",COUNTA($A$8:A13))</f>
       </c>
-      <c r="C13" s="55"/>
+      <c r="C13" s="56"/>
       <c r="D13" s="70"/>
       <c r="E13" s="10"/>
-      <c r="F13" s="53"/>
+      <c r="F13" s="54"/>
       <c r="G13" s="70"/>
       <c r="H13" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
-      <c r="A14" s="51"/>
-      <c r="B14" s="56">
+      <c r="A14" s="52"/>
+      <c r="B14" s="57">
         <f>IF(A14="","",COUNTA($A$8:A14))</f>
       </c>
-      <c r="C14" s="56"/>
+      <c r="C14" s="57"/>
       <c r="D14" s="69"/>
       <c r="E14" s="7"/>
-      <c r="F14" s="51"/>
+      <c r="F14" s="52"/>
       <c r="G14" s="69"/>
       <c r="H14" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
-      <c r="A15" s="53"/>
-      <c r="B15" s="55">
+      <c r="A15" s="54"/>
+      <c r="B15" s="56">
         <f>IF(A15="","",COUNTA($A$8:A15))</f>
       </c>
-      <c r="C15" s="55"/>
+      <c r="C15" s="56"/>
       <c r="D15" s="70"/>
       <c r="E15" s="10"/>
-      <c r="F15" s="53"/>
+      <c r="F15" s="54"/>
       <c r="G15" s="70"/>
       <c r="H15" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
-      <c r="A16" s="51"/>
-      <c r="B16" s="56">
+      <c r="A16" s="52"/>
+      <c r="B16" s="57">
         <f>IF(A16="","",COUNTA($A$8:A16))</f>
       </c>
-      <c r="C16" s="56"/>
+      <c r="C16" s="57"/>
       <c r="D16" s="69"/>
       <c r="E16" s="7"/>
-      <c r="F16" s="51"/>
+      <c r="F16" s="52"/>
       <c r="G16" s="69"/>
       <c r="H16" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
-      <c r="A17" s="53"/>
-      <c r="B17" s="55">
+      <c r="A17" s="54"/>
+      <c r="B17" s="56">
         <f>IF(A17="","",COUNTA($A$8:A17))</f>
       </c>
-      <c r="C17" s="55"/>
+      <c r="C17" s="56"/>
       <c r="D17" s="70"/>
       <c r="E17" s="10"/>
-      <c r="F17" s="53"/>
+      <c r="F17" s="54"/>
       <c r="G17" s="70"/>
       <c r="H17" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
-      <c r="A18" s="51"/>
-      <c r="B18" s="56">
+      <c r="A18" s="52"/>
+      <c r="B18" s="57">
         <f>IF(A18="","",COUNTA($A$8:A18))</f>
       </c>
-      <c r="C18" s="56"/>
+      <c r="C18" s="57"/>
       <c r="D18" s="69"/>
       <c r="E18" s="7"/>
-      <c r="F18" s="51"/>
+      <c r="F18" s="52"/>
       <c r="G18" s="69"/>
       <c r="H18" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="21.75">
-      <c r="A19" s="53"/>
-      <c r="B19" s="55">
+      <c r="A19" s="54"/>
+      <c r="B19" s="56">
         <f>IF(A19="","",COUNTA($A$8:A19))</f>
       </c>
-      <c r="C19" s="55"/>
+      <c r="C19" s="56"/>
       <c r="D19" s="70"/>
       <c r="E19" s="10"/>
-      <c r="F19" s="53"/>
+      <c r="F19" s="54"/>
       <c r="G19" s="70"/>
       <c r="H19" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="21.75">
-      <c r="A20" s="51"/>
-      <c r="B20" s="56">
+      <c r="A20" s="52"/>
+      <c r="B20" s="57">
         <f>IF(A20="","",COUNTA($A$8:A20))</f>
       </c>
-      <c r="C20" s="56"/>
+      <c r="C20" s="57"/>
       <c r="D20" s="69"/>
       <c r="E20" s="7"/>
-      <c r="F20" s="51"/>
+      <c r="F20" s="52"/>
       <c r="G20" s="69"/>
       <c r="H20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="21.75">
-      <c r="A21" s="53"/>
-      <c r="B21" s="55">
+      <c r="A21" s="54"/>
+      <c r="B21" s="56">
         <f>IF(A21="","",COUNTA($A$8:A21))</f>
       </c>
-      <c r="C21" s="55"/>
+      <c r="C21" s="56"/>
       <c r="D21" s="70"/>
       <c r="E21" s="10"/>
-      <c r="F21" s="53"/>
+      <c r="F21" s="54"/>
       <c r="G21" s="70"/>
       <c r="H21" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="21.75">
-      <c r="A22" s="51"/>
-      <c r="B22" s="56">
+      <c r="A22" s="52"/>
+      <c r="B22" s="57">
         <f>IF(A22="","",COUNTA($A$8:A22))</f>
       </c>
-      <c r="C22" s="56"/>
+      <c r="C22" s="57"/>
       <c r="D22" s="69"/>
       <c r="E22" s="7"/>
-      <c r="F22" s="51"/>
+      <c r="F22" s="52"/>
       <c r="G22" s="69"/>
       <c r="H22" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="21.75">
-      <c r="A23" s="53"/>
-      <c r="B23" s="55">
+      <c r="A23" s="54"/>
+      <c r="B23" s="56">
         <f>IF(A23="","",COUNTA($A$8:A23))</f>
       </c>
-      <c r="C23" s="55"/>
+      <c r="C23" s="56"/>
       <c r="D23" s="70"/>
       <c r="E23" s="10"/>
-      <c r="F23" s="53"/>
+      <c r="F23" s="54"/>
       <c r="G23" s="70"/>
       <c r="H23" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
-      <c r="A24" s="51"/>
-      <c r="B24" s="56">
+      <c r="A24" s="52"/>
+      <c r="B24" s="57">
         <f>IF(A24="","",COUNTA($A$8:A24))</f>
       </c>
-      <c r="C24" s="56"/>
+      <c r="C24" s="57"/>
       <c r="D24" s="69"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="51"/>
+      <c r="F24" s="52"/>
       <c r="G24" s="69"/>
       <c r="H24" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
-      <c r="A25" s="53"/>
-      <c r="B25" s="55">
+      <c r="A25" s="54"/>
+      <c r="B25" s="56">
         <f>IF(A25="","",COUNTA($A$8:A25))</f>
       </c>
-      <c r="C25" s="55"/>
+      <c r="C25" s="56"/>
       <c r="D25" s="70"/>
       <c r="E25" s="10"/>
-      <c r="F25" s="53"/>
+      <c r="F25" s="54"/>
       <c r="G25" s="70"/>
       <c r="H25" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21.75">
-      <c r="A26" s="51"/>
-      <c r="B26" s="56">
+      <c r="A26" s="52"/>
+      <c r="B26" s="57">
         <f>IF(A26="","",COUNTA($A$8:A26))</f>
       </c>
-      <c r="C26" s="56"/>
+      <c r="C26" s="57"/>
       <c r="D26" s="69"/>
       <c r="E26" s="7"/>
-      <c r="F26" s="51"/>
+      <c r="F26" s="52"/>
       <c r="G26" s="69"/>
       <c r="H26" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21.75">
-      <c r="A27" s="53"/>
-      <c r="B27" s="55">
+      <c r="A27" s="54"/>
+      <c r="B27" s="56">
         <f>IF(A27="","",COUNTA($A$8:A27))</f>
       </c>
-      <c r="C27" s="55"/>
+      <c r="C27" s="56"/>
       <c r="D27" s="70"/>
       <c r="E27" s="10"/>
-      <c r="F27" s="53"/>
+      <c r="F27" s="54"/>
       <c r="G27" s="70"/>
       <c r="H27" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="21.75">
-      <c r="A28" s="51"/>
-      <c r="B28" s="56">
+      <c r="A28" s="52"/>
+      <c r="B28" s="57">
         <f>IF(A28="","",COUNTA($A$8:A28))</f>
       </c>
-      <c r="C28" s="56"/>
+      <c r="C28" s="57"/>
       <c r="D28" s="69"/>
       <c r="E28" s="7"/>
-      <c r="F28" s="51"/>
+      <c r="F28" s="52"/>
       <c r="G28" s="69"/>
       <c r="H28" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="21.75">
-      <c r="A29" s="53"/>
-      <c r="B29" s="55">
+      <c r="A29" s="54"/>
+      <c r="B29" s="56">
         <f>IF(A29="","",COUNTA($A$8:A29))</f>
       </c>
-      <c r="C29" s="55"/>
+      <c r="C29" s="56"/>
       <c r="D29" s="70"/>
       <c r="E29" s="10"/>
-      <c r="F29" s="53"/>
+      <c r="F29" s="54"/>
       <c r="G29" s="70"/>
       <c r="H29" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="21.75">
-      <c r="A30" s="51"/>
-      <c r="B30" s="56">
+      <c r="A30" s="52"/>
+      <c r="B30" s="57">
         <f>IF(A30="","",COUNTA($A$8:A30))</f>
       </c>
-      <c r="C30" s="56"/>
+      <c r="C30" s="57"/>
       <c r="D30" s="69"/>
       <c r="E30" s="7"/>
-      <c r="F30" s="51"/>
+      <c r="F30" s="52"/>
       <c r="G30" s="69"/>
       <c r="H30" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="21.75">
-      <c r="A31" s="53"/>
-      <c r="B31" s="55">
+      <c r="A31" s="54"/>
+      <c r="B31" s="56">
         <f>IF(A31="","",COUNTA($A$8:A31))</f>
       </c>
-      <c r="C31" s="55"/>
+      <c r="C31" s="56"/>
       <c r="D31" s="70"/>
       <c r="E31" s="10"/>
-      <c r="F31" s="53"/>
+      <c r="F31" s="54"/>
       <c r="G31" s="70"/>
       <c r="H31" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="21.75">
-      <c r="A32" s="51"/>
-      <c r="B32" s="56">
+      <c r="A32" s="52"/>
+      <c r="B32" s="57">
         <f>IF(A32="","",COUNTA($A$8:A32))</f>
       </c>
-      <c r="C32" s="56"/>
+      <c r="C32" s="57"/>
       <c r="D32" s="69"/>
       <c r="E32" s="7"/>
-      <c r="F32" s="51"/>
+      <c r="F32" s="52"/>
       <c r="G32" s="69"/>
       <c r="H32" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="21.75">
-      <c r="A33" s="53"/>
-      <c r="B33" s="55">
+      <c r="A33" s="54"/>
+      <c r="B33" s="56">
         <f>IF(A33="","",COUNTA($A$8:A33))</f>
       </c>
-      <c r="C33" s="55"/>
+      <c r="C33" s="56"/>
       <c r="D33" s="70"/>
       <c r="E33" s="10"/>
-      <c r="F33" s="53"/>
+      <c r="F33" s="54"/>
       <c r="G33" s="70"/>
       <c r="H33" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="21.75">
-      <c r="A34" s="51"/>
-      <c r="B34" s="56">
+      <c r="A34" s="52"/>
+      <c r="B34" s="57">
         <f>IF(A34="","",COUNTA($A$8:A34))</f>
       </c>
-      <c r="C34" s="56"/>
+      <c r="C34" s="57"/>
       <c r="D34" s="69"/>
       <c r="E34" s="7"/>
-      <c r="F34" s="51"/>
+      <c r="F34" s="52"/>
       <c r="G34" s="69"/>
       <c r="H34" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="21.75">
-      <c r="A35" s="53"/>
-      <c r="B35" s="55">
+      <c r="A35" s="54"/>
+      <c r="B35" s="56">
         <f>IF(A35="","",COUNTA($A$8:A35))</f>
       </c>
-      <c r="C35" s="55"/>
+      <c r="C35" s="56"/>
       <c r="D35" s="70"/>
       <c r="E35" s="10"/>
-      <c r="F35" s="53"/>
+      <c r="F35" s="54"/>
       <c r="G35" s="70"/>
       <c r="H35" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="21.75">
-      <c r="A36" s="51"/>
-      <c r="B36" s="56">
+      <c r="A36" s="52"/>
+      <c r="B36" s="57">
         <f>IF(A36="","",COUNTA($A$8:A36))</f>
       </c>
-      <c r="C36" s="56"/>
+      <c r="C36" s="57"/>
       <c r="D36" s="69"/>
       <c r="E36" s="7"/>
-      <c r="F36" s="51"/>
+      <c r="F36" s="52"/>
       <c r="G36" s="69"/>
       <c r="H36" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="21.75">
-      <c r="A37" s="53"/>
-      <c r="B37" s="55">
+      <c r="A37" s="54"/>
+      <c r="B37" s="56">
         <f>IF(A37="","",COUNTA($A$8:A37))</f>
       </c>
-      <c r="C37" s="55"/>
+      <c r="C37" s="56"/>
       <c r="D37" s="70"/>
       <c r="E37" s="10"/>
-      <c r="F37" s="53"/>
+      <c r="F37" s="54"/>
       <c r="G37" s="70"/>
       <c r="H37" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="21.75">
-      <c r="A38" s="51"/>
-      <c r="B38" s="56">
+      <c r="A38" s="52"/>
+      <c r="B38" s="57">
         <f>IF(A38="","",COUNTA($A$8:A38))</f>
       </c>
-      <c r="C38" s="56"/>
+      <c r="C38" s="57"/>
       <c r="D38" s="69"/>
       <c r="E38" s="7"/>
-      <c r="F38" s="51"/>
+      <c r="F38" s="52"/>
       <c r="G38" s="69"/>
       <c r="H38" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="21.75">
-      <c r="A39" s="53"/>
-      <c r="B39" s="55">
+      <c r="A39" s="54"/>
+      <c r="B39" s="56">
         <f>IF(A39="","",COUNTA($A$8:A39))</f>
       </c>
-      <c r="C39" s="55"/>
+      <c r="C39" s="56"/>
       <c r="D39" s="70"/>
       <c r="E39" s="10"/>
-      <c r="F39" s="53"/>
+      <c r="F39" s="54"/>
       <c r="G39" s="70"/>
       <c r="H39" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="21.75">
-      <c r="A40" s="51"/>
-      <c r="B40" s="56">
+      <c r="A40" s="52"/>
+      <c r="B40" s="57">
         <f>IF(A40="","",COUNTA($A$8:A40))</f>
       </c>
-      <c r="C40" s="56"/>
+      <c r="C40" s="57"/>
       <c r="D40" s="69"/>
       <c r="E40" s="7"/>
-      <c r="F40" s="51"/>
+      <c r="F40" s="52"/>
       <c r="G40" s="69"/>
       <c r="H40" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="21.75">
-      <c r="A41" s="53"/>
-      <c r="B41" s="55">
+      <c r="A41" s="54"/>
+      <c r="B41" s="56">
         <f>IF(A41="","",COUNTA($A$8:A41))</f>
       </c>
-      <c r="C41" s="55"/>
+      <c r="C41" s="56"/>
       <c r="D41" s="70"/>
       <c r="E41" s="10"/>
-      <c r="F41" s="53"/>
+      <c r="F41" s="54"/>
       <c r="G41" s="70"/>
       <c r="H41" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="21.75">
-      <c r="A42" s="51"/>
-      <c r="B42" s="56">
+      <c r="A42" s="52"/>
+      <c r="B42" s="57">
         <f>IF(A42="","",COUNTA($A$8:A42))</f>
       </c>
-      <c r="C42" s="56"/>
+      <c r="C42" s="57"/>
       <c r="D42" s="69"/>
       <c r="E42" s="7"/>
-      <c r="F42" s="51"/>
+      <c r="F42" s="52"/>
       <c r="G42" s="69"/>
       <c r="H42" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="21.75">
-      <c r="A43" s="53"/>
-      <c r="B43" s="55">
+      <c r="A43" s="54"/>
+      <c r="B43" s="56">
         <f>IF(A43="","",COUNTA($A$8:A43))</f>
       </c>
-      <c r="C43" s="55"/>
+      <c r="C43" s="56"/>
       <c r="D43" s="70"/>
       <c r="E43" s="10"/>
-      <c r="F43" s="53"/>
+      <c r="F43" s="54"/>
       <c r="G43" s="70"/>
       <c r="H43" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="21.75">
-      <c r="A44" s="51"/>
-      <c r="B44" s="56">
+      <c r="A44" s="52"/>
+      <c r="B44" s="57">
         <f>IF(A44="","",COUNTA($A$8:A44))</f>
       </c>
-      <c r="C44" s="56"/>
+      <c r="C44" s="57"/>
       <c r="D44" s="69"/>
       <c r="E44" s="7"/>
-      <c r="F44" s="51"/>
+      <c r="F44" s="52"/>
       <c r="G44" s="69"/>
       <c r="H44" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="21.75">
-      <c r="A45" s="53"/>
-      <c r="B45" s="55">
+      <c r="A45" s="54"/>
+      <c r="B45" s="56">
         <f>IF(A45="","",COUNTA($A$8:A45))</f>
       </c>
-      <c r="C45" s="55"/>
+      <c r="C45" s="56"/>
       <c r="D45" s="70"/>
       <c r="E45" s="10"/>
-      <c r="F45" s="53"/>
+      <c r="F45" s="54"/>
       <c r="G45" s="70"/>
       <c r="H45" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="21.75">
-      <c r="A46" s="51"/>
-      <c r="B46" s="56">
+      <c r="A46" s="52"/>
+      <c r="B46" s="57">
         <f>IF(A46="","",COUNTA($A$8:A46))</f>
       </c>
-      <c r="C46" s="56"/>
+      <c r="C46" s="57"/>
       <c r="D46" s="69"/>
       <c r="E46" s="7"/>
-      <c r="F46" s="51"/>
+      <c r="F46" s="52"/>
       <c r="G46" s="69"/>
       <c r="H46" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="21.75">
-      <c r="A47" s="53"/>
-      <c r="B47" s="55">
+      <c r="A47" s="54"/>
+      <c r="B47" s="56">
         <f>IF(A47="","",COUNTA($A$8:A47))</f>
       </c>
-      <c r="C47" s="55"/>
+      <c r="C47" s="56"/>
       <c r="D47" s="70"/>
       <c r="E47" s="10"/>
-      <c r="F47" s="53"/>
+      <c r="F47" s="54"/>
       <c r="G47" s="70"/>
       <c r="H47" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="21.75">
       <c r="A48" s="13"/>
-      <c r="B48" s="29"/>
-      <c r="C48" s="29"/>
-      <c r="D48" s="40"/>
+      <c r="B48" s="30"/>
+      <c r="C48" s="30"/>
+      <c r="D48" s="41"/>
       <c r="E48" s="13"/>
       <c r="F48" s="65"/>
-      <c r="G48" s="40"/>
+      <c r="G48" s="41"/>
       <c r="H48" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="21.75">
       <c r="A49" s="13"/>
-      <c r="B49" s="29"/>
-      <c r="C49" s="29"/>
-      <c r="D49" s="40"/>
+      <c r="B49" s="30"/>
+      <c r="C49" s="30"/>
+      <c r="D49" s="41"/>
       <c r="E49" s="13"/>
       <c r="F49" s="65"/>
-      <c r="G49" s="40"/>
+      <c r="G49" s="41"/>
       <c r="H49" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="21.75">
       <c r="A50" s="19" t="s">
-        <v>254</v>
-      </c>
-      <c r="B50" s="36"/>
-      <c r="C50" s="36"/>
+        <v>258</v>
+      </c>
+      <c r="B50" s="37"/>
+      <c r="C50" s="37"/>
       <c r="D50" s="71"/>
       <c r="E50" s="19"/>
       <c r="F50" s="72"/>
@@ -3864,8 +3875,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" style="12" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="57" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="12" width="36.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="38" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="59.005" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="12" width="36.005" customWidth="1" bestFit="1"/>
     <col min="5" max="5" style="12" width="23.14785714285714" customWidth="1" bestFit="1"/>
     <col min="6" max="6" style="12" width="28.290714285714284" customWidth="1" bestFit="1"/>
@@ -3876,7 +3887,7 @@
       <c r="A1" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="25"/>
+      <c r="B1" s="26"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
@@ -3887,7 +3898,7 @@
       <c r="A2" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="B2" s="26"/>
+      <c r="B2" s="27"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -3895,31 +3906,31 @@
       <c r="G2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="42" t="s">
         <v>212</v>
       </c>
-      <c r="B3" s="50" t="s">
+      <c r="B3" s="51" t="s">
         <v>213</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="42" t="s">
         <v>214</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="E3" s="41" t="s">
+      <c r="E3" s="42" t="s">
         <v>216</v>
       </c>
-      <c r="F3" s="41" t="s">
+      <c r="F3" s="42" t="s">
         <v>217</v>
       </c>
-      <c r="G3" s="41" t="s">
+      <c r="G3" s="42" t="s">
         <v>218</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="66.75">
-      <c r="A4" s="51"/>
-      <c r="B4" s="52">
+      <c r="A4" s="52"/>
+      <c r="B4" s="53">
         <v>1</v>
       </c>
       <c r="C4" s="7" t="s">
@@ -3937,8 +3948,8 @@
       <c r="G4" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="88.5">
-      <c r="A5" s="53"/>
-      <c r="B5" s="54">
+      <c r="A5" s="54"/>
+      <c r="B5" s="55">
         <v>2</v>
       </c>
       <c r="C5" s="10" t="s">
@@ -3955,26 +3966,28 @@
       </c>
       <c r="G5" s="10"/>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
-      <c r="A6" s="51"/>
-      <c r="B6" s="52">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="54.75">
+      <c r="A6" s="52"/>
+      <c r="B6" s="53">
         <v>3</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="D6" s="7"/>
+      <c r="D6" s="7" t="s">
+        <v>228</v>
+      </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
-      <c r="A7" s="53"/>
-      <c r="B7" s="54">
+      <c r="A7" s="54"/>
+      <c r="B7" s="55">
         <v>4</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
@@ -3982,12 +3995,12 @@
       <c r="G7" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
-      <c r="A8" s="51"/>
-      <c r="B8" s="52">
+      <c r="A8" s="52"/>
+      <c r="B8" s="53">
         <v>5</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
@@ -3995,12 +4008,12 @@
       <c r="G8" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="53"/>
-      <c r="B9" s="54">
+      <c r="A9" s="54"/>
+      <c r="B9" s="55">
         <v>6</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -4008,12 +4021,12 @@
       <c r="G9" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
-      <c r="A10" s="51"/>
-      <c r="B10" s="52">
+      <c r="A10" s="52"/>
+      <c r="B10" s="53">
         <v>7</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="7"/>
@@ -4021,12 +4034,12 @@
       <c r="G10" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
-      <c r="A11" s="53"/>
-      <c r="B11" s="54">
+      <c r="A11" s="54"/>
+      <c r="B11" s="55">
         <v>8</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
@@ -4034,12 +4047,12 @@
       <c r="G11" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
-      <c r="A12" s="51"/>
-      <c r="B12" s="52">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53">
         <v>9</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
@@ -4047,12 +4060,12 @@
       <c r="G12" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="53"/>
-      <c r="B13" s="54">
+      <c r="A13" s="54"/>
+      <c r="B13" s="55">
         <v>10</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
@@ -4060,12 +4073,12 @@
       <c r="G13" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
-      <c r="A14" s="51"/>
-      <c r="B14" s="52">
+      <c r="A14" s="52"/>
+      <c r="B14" s="53">
         <v>11</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="7"/>
@@ -4073,12 +4086,12 @@
       <c r="G14" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
-      <c r="A15" s="53"/>
-      <c r="B15" s="54">
+      <c r="A15" s="54"/>
+      <c r="B15" s="55">
         <v>12</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D15" s="10"/>
       <c r="E15" s="10"/>
@@ -4086,12 +4099,12 @@
       <c r="G15" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
-      <c r="A16" s="51"/>
-      <c r="B16" s="52">
+      <c r="A16" s="52"/>
+      <c r="B16" s="53">
         <v>13</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
@@ -4099,12 +4112,12 @@
       <c r="G16" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
-      <c r="A17" s="53"/>
-      <c r="B17" s="54">
+      <c r="A17" s="54"/>
+      <c r="B17" s="55">
         <v>14</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
@@ -4112,12 +4125,12 @@
       <c r="G17" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
-      <c r="A18" s="51"/>
-      <c r="B18" s="52">
+      <c r="A18" s="52"/>
+      <c r="B18" s="53">
         <v>15</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
@@ -4125,8 +4138,8 @@
       <c r="G18" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="21.75">
-      <c r="A19" s="53"/>
-      <c r="B19" s="55"/>
+      <c r="A19" s="54"/>
+      <c r="B19" s="56"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
@@ -4134,8 +4147,8 @@
       <c r="G19" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="21.75">
-      <c r="A20" s="51"/>
-      <c r="B20" s="56"/>
+      <c r="A20" s="52"/>
+      <c r="B20" s="57"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
@@ -4143,8 +4156,8 @@
       <c r="G20" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="21.75">
-      <c r="A21" s="53"/>
-      <c r="B21" s="55"/>
+      <c r="A21" s="54"/>
+      <c r="B21" s="56"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
@@ -4152,8 +4165,8 @@
       <c r="G21" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="21.75">
-      <c r="A22" s="51"/>
-      <c r="B22" s="56"/>
+      <c r="A22" s="52"/>
+      <c r="B22" s="57"/>
       <c r="C22" s="7"/>
       <c r="D22" s="7"/>
       <c r="E22" s="7"/>
@@ -4161,8 +4174,8 @@
       <c r="G22" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="21.75">
-      <c r="A23" s="53"/>
-      <c r="B23" s="55"/>
+      <c r="A23" s="54"/>
+      <c r="B23" s="56"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
@@ -4170,8 +4183,8 @@
       <c r="G23" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
-      <c r="A24" s="51"/>
-      <c r="B24" s="56"/>
+      <c r="A24" s="52"/>
+      <c r="B24" s="57"/>
       <c r="C24" s="7"/>
       <c r="D24" s="7"/>
       <c r="E24" s="7"/>
@@ -4179,8 +4192,8 @@
       <c r="G24" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
-      <c r="A25" s="53"/>
-      <c r="B25" s="55"/>
+      <c r="A25" s="54"/>
+      <c r="B25" s="56"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
@@ -4188,8 +4201,8 @@
       <c r="G25" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21.75">
-      <c r="A26" s="51"/>
-      <c r="B26" s="56"/>
+      <c r="A26" s="52"/>
+      <c r="B26" s="57"/>
       <c r="C26" s="7"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
@@ -4197,8 +4210,8 @@
       <c r="G26" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21.75">
-      <c r="A27" s="53"/>
-      <c r="B27" s="55"/>
+      <c r="A27" s="54"/>
+      <c r="B27" s="56"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
@@ -4206,8 +4219,8 @@
       <c r="G27" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="21.75">
-      <c r="A28" s="51"/>
-      <c r="B28" s="56"/>
+      <c r="A28" s="52"/>
+      <c r="B28" s="57"/>
       <c r="C28" s="7"/>
       <c r="D28" s="7"/>
       <c r="E28" s="7"/>
@@ -4215,8 +4228,8 @@
       <c r="G28" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="21.75">
-      <c r="A29" s="53"/>
-      <c r="B29" s="55"/>
+      <c r="A29" s="54"/>
+      <c r="B29" s="56"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
@@ -4224,8 +4237,8 @@
       <c r="G29" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="21.75">
-      <c r="A30" s="51"/>
-      <c r="B30" s="56"/>
+      <c r="A30" s="52"/>
+      <c r="B30" s="57"/>
       <c r="C30" s="7"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
@@ -4233,8 +4246,8 @@
       <c r="G30" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="21.75">
-      <c r="A31" s="53"/>
-      <c r="B31" s="55"/>
+      <c r="A31" s="54"/>
+      <c r="B31" s="56"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -4242,8 +4255,8 @@
       <c r="G31" s="10"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="21.75">
-      <c r="A32" s="51"/>
-      <c r="B32" s="56"/>
+      <c r="A32" s="52"/>
+      <c r="B32" s="57"/>
       <c r="C32" s="7"/>
       <c r="D32" s="7"/>
       <c r="E32" s="7"/>
@@ -4251,8 +4264,8 @@
       <c r="G32" s="7"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="21.75">
-      <c r="A33" s="53"/>
-      <c r="B33" s="55"/>
+      <c r="A33" s="54"/>
+      <c r="B33" s="56"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
@@ -4276,14 +4289,14 @@
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="8.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="40.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="32.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="49" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="20" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="8.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="40.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="32.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="50" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="28.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
@@ -4295,7 +4308,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="F1" s="1"/>
-      <c r="G1" s="38"/>
+      <c r="G1" s="39"/>
       <c r="H1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
@@ -4307,7 +4320,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="39"/>
+      <c r="G2" s="40"/>
       <c r="H2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
@@ -4317,7 +4330,7 @@
       <c r="D3" s="13"/>
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
-      <c r="G3" s="40"/>
+      <c r="G3" s="41"/>
       <c r="H3" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
@@ -4327,7 +4340,7 @@
       <c r="D4" s="13"/>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
-      <c r="G4" s="40"/>
+      <c r="G4" s="41"/>
       <c r="H4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
@@ -4337,7 +4350,7 @@
       <c r="D5" s="13"/>
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
-      <c r="G5" s="40"/>
+      <c r="G5" s="41"/>
       <c r="H5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
@@ -4347,32 +4360,32 @@
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
-      <c r="G6" s="40"/>
+      <c r="G6" s="41"/>
       <c r="H6" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="42" t="s">
         <v>185</v>
       </c>
-      <c r="B7" s="41" t="s">
+      <c r="B7" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="C7" s="41" t="s">
+      <c r="C7" s="42" t="s">
         <v>187</v>
       </c>
-      <c r="D7" s="41" t="s">
+      <c r="D7" s="42" t="s">
         <v>188</v>
       </c>
-      <c r="E7" s="41" t="s">
+      <c r="E7" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="F7" s="41" t="s">
+      <c r="F7" s="42" t="s">
         <v>190</v>
       </c>
-      <c r="G7" s="42" t="s">
+      <c r="G7" s="43" t="s">
         <v>191</v>
       </c>
-      <c r="H7" s="41" t="s">
+      <c r="H7" s="42" t="s">
         <v>144</v>
       </c>
     </row>
@@ -4395,7 +4408,7 @@
       <c r="F8" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="44">
         <f>SUMIF(&amp;apos;Session Log&amp;apos;!C8:C200,A8,&amp;apos;Session Log&amp;apos;!G8:G200)</f>
       </c>
       <c r="H8" s="13"/>
@@ -4419,7 +4432,7 @@
       <c r="F9" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="G9" s="43">
+      <c r="G9" s="44">
         <f>SUMIF(&amp;apos;Session Log&amp;apos;!C8:C200,A9,&amp;apos;Session Log&amp;apos;!G8:G200)</f>
       </c>
       <c r="H9" s="13"/>
@@ -4443,7 +4456,7 @@
       <c r="F10" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="G10" s="43">
+      <c r="G10" s="44">
         <f>SUMIF(&amp;apos;Session Log&amp;apos;!C8:C200,A10,&amp;apos;Session Log&amp;apos;!G8:G200)</f>
       </c>
       <c r="H10" s="13"/>
@@ -4467,7 +4480,7 @@
       <c r="F11" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="G11" s="43">
+      <c r="G11" s="44">
         <f>SUMIF(&amp;apos;Session Log&amp;apos;!C8:C200,A11,&amp;apos;Session Log&amp;apos;!G8:G200)</f>
       </c>
       <c r="H11" s="13"/>
@@ -4479,52 +4492,52 @@
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
-      <c r="G12" s="40"/>
+      <c r="G12" s="41"/>
       <c r="H12" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="44" t="s">
+      <c r="A13" s="45" t="s">
         <v>208</v>
       </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="45"/>
-      <c r="H13" s="44"/>
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+      <c r="D13" s="45"/>
+      <c r="E13" s="45"/>
+      <c r="F13" s="45"/>
+      <c r="G13" s="46"/>
+      <c r="H13" s="45"/>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
-      <c r="A14" s="46" t="s">
+      <c r="A14" s="47" t="s">
         <v>209</v>
       </c>
-      <c r="B14" s="47"/>
-      <c r="C14" s="47"/>
-      <c r="D14" s="47"/>
-      <c r="E14" s="47"/>
-      <c r="F14" s="47"/>
-      <c r="G14" s="48"/>
-      <c r="H14" s="47"/>
+      <c r="B14" s="48"/>
+      <c r="C14" s="48"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="48"/>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
-      <c r="A15" s="47"/>
-      <c r="B15" s="47"/>
-      <c r="C15" s="47"/>
-      <c r="D15" s="47"/>
-      <c r="E15" s="47"/>
-      <c r="F15" s="47"/>
-      <c r="G15" s="48"/>
-      <c r="H15" s="47"/>
+      <c r="A15" s="48"/>
+      <c r="B15" s="48"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="48"/>
+      <c r="E15" s="48"/>
+      <c r="F15" s="48"/>
+      <c r="G15" s="49"/>
+      <c r="H15" s="48"/>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
-      <c r="A16" s="47"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
-      <c r="D16" s="47"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="48"/>
-      <c r="H16" s="47"/>
+      <c r="A16" s="48"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
+      <c r="D16" s="48"/>
+      <c r="E16" s="48"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4545,18 +4558,18 @@
   <dimension ref="A1:H27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="37" width="10.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="22.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="20" width="32.005" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="20" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="38" width="10.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="32.005" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="12" width="14.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="26" t="s">
         <v>135</v>
       </c>
       <c r="B1" s="1"/>
@@ -4568,7 +4581,7 @@
       <c r="H1" s="1"/>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="21.75">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="27" t="s">
         <v>136</v>
       </c>
       <c r="B2" s="2"/>
@@ -4580,19 +4593,19 @@
       <c r="H2" s="2"/>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="21.75">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="B3" s="28"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
-      <c r="A4" s="29"/>
+      <c r="A4" s="30"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
@@ -4602,7 +4615,7 @@
       <c r="H4" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
-      <c r="A5" s="29"/>
+      <c r="A5" s="30"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
@@ -4612,7 +4625,7 @@
       <c r="H5" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
-      <c r="A6" s="29"/>
+      <c r="A6" s="30"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
@@ -4622,7 +4635,7 @@
       <c r="H6" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="31" t="s">
         <v>138</v>
       </c>
       <c r="B7" s="14" t="s">
@@ -4648,7 +4661,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="21.75">
-      <c r="A8" s="31">
+      <c r="A8" s="32">
         <v>2</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -4668,7 +4681,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="21.75">
-      <c r="A9" s="32">
+      <c r="A9" s="33">
         <v>3</v>
       </c>
       <c r="B9" s="10" t="s">
@@ -4688,7 +4701,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="21.75">
-      <c r="A10" s="31">
+      <c r="A10" s="32">
         <v>17</v>
       </c>
       <c r="B10" s="7" t="s">
@@ -4708,7 +4721,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="21.75">
-      <c r="A11" s="32">
+      <c r="A11" s="33">
         <v>18</v>
       </c>
       <c r="B11" s="10" t="s">
@@ -4728,7 +4741,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="21.75">
-      <c r="A12" s="31">
+      <c r="A12" s="32">
         <v>27</v>
       </c>
       <c r="B12" s="7" t="s">
@@ -4746,7 +4759,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="21.75">
-      <c r="A13" s="32">
+      <c r="A13" s="33">
         <v>22</v>
       </c>
       <c r="B13" s="10" t="s">
@@ -4764,7 +4777,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="21.75">
-      <c r="A14" s="31">
+      <c r="A14" s="32">
         <v>21</v>
       </c>
       <c r="B14" s="7" t="s">
@@ -4784,7 +4797,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="21.75">
-      <c r="A15" s="32">
+      <c r="A15" s="33">
         <v>20</v>
       </c>
       <c r="B15" s="10" t="s">
@@ -4802,7 +4815,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="21.75">
-      <c r="A16" s="31">
+      <c r="A16" s="32">
         <v>16</v>
       </c>
       <c r="B16" s="7" t="s">
@@ -4820,7 +4833,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="21.75">
-      <c r="A17" s="32">
+      <c r="A17" s="33">
         <v>23</v>
       </c>
       <c r="B17" s="10" t="s">
@@ -4838,7 +4851,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="21.75">
-      <c r="A18" s="31">
+      <c r="A18" s="32">
         <v>24</v>
       </c>
       <c r="B18" s="7" t="s">
@@ -4856,7 +4869,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="21.75">
-      <c r="A19" s="32">
+      <c r="A19" s="33">
         <v>12</v>
       </c>
       <c r="B19" s="10" t="s">
@@ -4876,7 +4889,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="21.75">
-      <c r="A20" s="31">
+      <c r="A20" s="32">
         <v>13</v>
       </c>
       <c r="B20" s="7" t="s">
@@ -4896,7 +4909,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="21.75">
-      <c r="A21" s="32">
+      <c r="A21" s="33">
         <v>19</v>
       </c>
       <c r="B21" s="10" t="s">
@@ -4914,29 +4927,29 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="21.75">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="34" t="s">
         <v>169</v>
       </c>
-      <c r="B22" s="34" t="s">
+      <c r="B22" s="35" t="s">
         <v>170</v>
       </c>
-      <c r="C22" s="34" t="s">
+      <c r="C22" s="35" t="s">
         <v>171</v>
       </c>
-      <c r="D22" s="34"/>
-      <c r="E22" s="35"/>
-      <c r="F22" s="35" t="s">
+      <c r="D22" s="35"/>
+      <c r="E22" s="36"/>
+      <c r="F22" s="36" t="s">
         <v>48</v>
       </c>
-      <c r="G22" s="34" t="s">
+      <c r="G22" s="35" t="s">
         <v>172</v>
       </c>
-      <c r="H22" s="35" t="s">
+      <c r="H22" s="36" t="s">
         <v>173</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="21.75">
-      <c r="A23" s="32" t="s">
+      <c r="A23" s="33" t="s">
         <v>174</v>
       </c>
       <c r="B23" s="10" t="s">
@@ -4958,7 +4971,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="32" t="s">
         <v>178</v>
       </c>
       <c r="B24" s="7" t="s">
@@ -4980,7 +4993,7 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
-      <c r="A25" s="29"/>
+      <c r="A25" s="30"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
@@ -4990,7 +5003,7 @@
       <c r="H25" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="21.75">
-      <c r="A26" s="29"/>
+      <c r="A26" s="30"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
@@ -5000,7 +5013,7 @@
       <c r="H26" s="13"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="21.75">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="37" t="s">
         <v>182</v>
       </c>
       <c r="B27" s="19"/>
@@ -5030,12 +5043,12 @@
   <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="36.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="16.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="20.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="36.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="36.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="16.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="20.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="25" width="36.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="25" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">
@@ -5063,32 +5076,32 @@
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="21.75">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="21.75">
       <c r="A5" s="13"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
       <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="21.75">
       <c r="A6" s="13"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
       <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="21.75">
       <c r="A7" s="5" t="s">
@@ -5295,16 +5308,16 @@
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="21.75">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
+      <c r="E24" s="20"/>
+      <c r="F24" s="20"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="21.75">
       <c r="A25" s="21" t="s">
@@ -5319,8 +5332,8 @@
       <c r="D25" s="24">
         <f>IF(COUNT(D8:D22)=0,"—",AVERAGE(D8:D22))</f>
       </c>
-      <c r="E25" s="13"/>
-      <c r="F25" s="13"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5339,13 +5352,13 @@
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="20" width="28.005" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="20" width="14.005" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="20" width="12.005" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="20" width="18.005" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="20" width="36.005" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="20" width="32.005" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="20" width="22.005" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="12" width="28.005" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="12" width="14.005" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="12" width="12.005" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="12" width="18.005" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="12" width="36.005" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="12" width="32.005" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="12" width="22.005" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="21.75">

</xml_diff>